<commit_message>
Add goal notes, Garmin Coach plans, and combined calendar
</commit_message>
<xml_diff>
--- a/templates/Training-example.xlsx
+++ b/templates/Training-example.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy" sheetId="1" r:id="R9a9312849e474d16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring" sheetId="2" r:id="R47ecf7517b594543"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="3" r:id="Rf2ef6c251baa4074"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy" sheetId="1" r:id="R4ca80f28de9b48c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring" sheetId="2" r:id="Ra6d092b3991541a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="3" r:id="R9088dd6b4a724988"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -703,7 +703,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -745,8 +745,18 @@
         <x:fgColor rgb="FFE8F3EC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E3EF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="104">
     <x:border diagonalUp="0" diagonalDown="0">
       <x:left/>
       <x:right/>
@@ -788,6 +798,1084 @@
       <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFB7C3CF"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="thin">
+        <x:color rgb="FFCCD6E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF8297AD"/>
       </x:bottom>
       <x:diagonal/>
     </x:border>
@@ -830,7 +1918,7 @@
     </x:xf>
     <x:xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="132">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -932,6 +2020,425 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="25" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="6" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="7" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="8" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="9" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="10" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="11" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="12" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="13" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="14" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="15" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="16" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="17" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="18" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="19" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="20" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="21" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="22" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="23" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="24" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="25" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="26" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="27" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="28" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="29" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="30" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="31" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="32" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="33" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="34" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="35" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="36" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="37" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="38" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="39" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="40" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="41" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="42" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="43" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="44" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="45" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="46" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="47" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="48" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="49" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="50" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="51" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="52" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="53" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="54" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="55" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="56" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="57" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="58" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="59" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="60" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="61" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="62" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="63" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="64" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="65" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="66" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="67" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="68" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="69" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="70" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="71" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="72" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="73" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="74" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="75" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="76" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="77" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="78" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="79" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="80" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="81" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="82" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="83" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="84" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="85" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="86" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="87" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="88" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="89" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="90" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="91" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="92" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="93" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="94" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="95" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="96" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="4" borderId="97" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="98" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="5" borderId="99" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="172" fontId="8" fillId="6" borderId="100" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="101" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="102" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="5" borderId="103" xfId="24" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -1318,11 +2825,11 @@
       <x:c r="D5" s="2"/>
       <x:c r="E5" s="2"/>
       <x:c r="F5" s="2"/>
-      <x:c r="G5" s="3"/>
-      <x:c r="H5" s="4"/>
+      <x:c r="G5" s="32"/>
+      <x:c r="H5" s="33"/>
       <x:c r="I5" s="4"/>
     </x:row>
-    <x:row r="6" ht="30" hidden="0" customHeight="1">
+    <x:row r="6" ht="36" hidden="0" customHeight="1">
       <x:c r="A6" s="5" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -1341,8 +2848,12 @@
       <x:c r="F6" s="5" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G6" s="3"/>
-      <x:c r="H6" s="4"/>
+      <x:c r="G6" s="31" t="str">
+        <x:v>result_column</x:v>
+      </x:c>
+      <x:c r="H6" s="31" t="str">
+        <x:v>garmin_types</x:v>
+      </x:c>
       <x:c r="I6" s="4"/>
     </x:row>
     <x:row r="7" ht="76" hidden="0" customHeight="1">
@@ -1364,8 +2875,10 @@
       <x:c r="F7" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="G7" s="3"/>
-      <x:c r="H7" s="4"/>
+      <x:c r="G7" s="29" t="str">
+        <x:v>Muscle-up result</x:v>
+      </x:c>
+      <x:c r="H7" s="30"/>
       <x:c r="I7" s="4"/>
     </x:row>
     <x:row r="8" ht="76" hidden="0" customHeight="1">
@@ -1387,8 +2900,10 @@
       <x:c r="F8" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="G8" s="3"/>
-      <x:c r="H8" s="4"/>
+      <x:c r="G8" s="29" t="str">
+        <x:v>HSPU result</x:v>
+      </x:c>
+      <x:c r="H8" s="30"/>
       <x:c r="I8" s="4"/>
     </x:row>
     <x:row r="9" ht="76" hidden="0" customHeight="1">
@@ -1410,8 +2925,10 @@
       <x:c r="F9" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="G9" s="3"/>
-      <x:c r="H9" s="4"/>
+      <x:c r="G9" s="29" t="str">
+        <x:v>Pistol result</x:v>
+      </x:c>
+      <x:c r="H9" s="30"/>
       <x:c r="I9" s="4"/>
     </x:row>
     <x:row r="10" ht="76" hidden="0" customHeight="1">
@@ -1433,19 +2950,35 @@
       <x:c r="F10" s="7" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="G10" s="3"/>
-      <x:c r="H10" s="4"/>
+      <x:c r="G10" s="29"/>
+      <x:c r="H10" s="30" t="str">
+        <x:v>running</x:v>
+      </x:c>
       <x:c r="I10" s="4"/>
     </x:row>
-    <x:row r="11" ht="18" hidden="0" customHeight="1">
-      <x:c r="A11" s="3"/>
-      <x:c r="B11" s="3"/>
-      <x:c r="C11" s="3"/>
-      <x:c r="D11" s="3"/>
-      <x:c r="E11" s="3"/>
-      <x:c r="F11" s="3"/>
-      <x:c r="G11" s="3"/>
-      <x:c r="H11" s="4"/>
+    <x:row r="11" ht="84" hidden="0" customHeight="1">
+      <x:c r="A11" s="26" t="str">
+        <x:v>swimming</x:v>
+      </x:c>
+      <x:c r="B11" s="27" t="str">
+        <x:v>Swimming</x:v>
+      </x:c>
+      <x:c r="C11" s="27" t="str">
+        <x:v>Maintain regular swimming</x:v>
+      </x:c>
+      <x:c r="D11" s="27" t="str">
+        <x:v>3 fixed 60 min guided swims/week; optional fourth (reported routine)</x:v>
+      </x:c>
+      <x:c r="E11" s="27" t="str">
+        <x:v>Record duration and distance for comparable swims</x:v>
+      </x:c>
+      <x:c r="F11" s="27" t="str">
+        <x:v>maintenance</x:v>
+      </x:c>
+      <x:c r="G11" s="29"/>
+      <x:c r="H11" s="30" t="str">
+        <x:v>swimming</x:v>
+      </x:c>
       <x:c r="I11" s="4"/>
     </x:row>
     <x:row r="12" ht="28" hidden="0" customHeight="1">
@@ -2860,15 +4393,18 @@
     <x:row r="1048575" ht="12.800000190734863" hidden="0"/>
     <x:row r="1048576" ht="12.800000190734863" hidden="0"/>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F7:F10">
       <x:formula1>"milestone,maintenance"</x:formula1>
       <x:formula2>0</x:formula2>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="F11">
+      <x:formula1>"milestone,maintenance"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb43341d1b50c4523"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3af5a92584f844ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2921,208 +4457,208 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="40" hidden="0" customHeight="1">
-      <x:c r="A3" s="17" t="s">
+      <x:c r="A3" s="34" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="B3" s="18"/>
-      <x:c r="C3" s="18"/>
-      <x:c r="D3" s="19" t="str">
+      <x:c r="B3" s="35"/>
+      <x:c r="C3" s="36"/>
+      <x:c r="D3" s="37" t="str">
         <x:f aca="0">IF(OR(B3="",C3=""),"",ROUND(MOD(C3-B3,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E3" s="7"/>
-      <x:c r="F3" s="7"/>
-      <x:c r="G3" s="7"/>
+      <x:c r="E3" s="38"/>
+      <x:c r="F3" s="39"/>
+      <x:c r="G3" s="40"/>
     </x:row>
     <x:row r="4" ht="40" hidden="0" customHeight="1">
-      <x:c r="A4" s="17" t="s">
+      <x:c r="A4" s="41" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="B4" s="20"/>
-      <x:c r="C4" s="20"/>
-      <x:c r="D4" s="19" t="str">
+      <x:c r="B4" s="42"/>
+      <x:c r="C4" s="43"/>
+      <x:c r="D4" s="44" t="str">
         <x:f aca="0">IF(OR(B4="",C4=""),"",ROUND(MOD(C4-B4,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E4" s="21"/>
-      <x:c r="F4" s="21"/>
-      <x:c r="G4" s="21"/>
+      <x:c r="E4" s="45"/>
+      <x:c r="F4" s="46"/>
+      <x:c r="G4" s="47"/>
     </x:row>
     <x:row r="5" ht="40" hidden="0" customHeight="1">
-      <x:c r="A5" s="17" t="s">
+      <x:c r="A5" s="48" t="s">
         <x:v>178</x:v>
       </x:c>
-      <x:c r="B5" s="18" t="n">
+      <x:c r="B5" s="49" t="n">
         <x:v>0.833333333333333</x:v>
       </x:c>
-      <x:c r="C5" s="18" t="n">
+      <x:c r="C5" s="50" t="n">
         <x:v>0.875</x:v>
       </x:c>
-      <x:c r="D5" s="19" t="n">
+      <x:c r="D5" s="51" t="n">
         <x:f aca="0">IF(OR(B5="",C5=""),"",ROUND(MOD(C5-B5,1)*1440,6))</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="E5" s="7" t="s">
+      <x:c r="E5" s="52" t="s">
         <x:v>179</x:v>
       </x:c>
-      <x:c r="F5" s="7" t="s">
+      <x:c r="F5" s="53" t="s">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="G5" s="7" t="s">
+      <x:c r="G5" s="54" t="s">
         <x:v>181</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="40" hidden="0" customHeight="1">
-      <x:c r="A6" s="17" t="s">
+      <x:c r="A6" s="55" t="s">
         <x:v>178</x:v>
       </x:c>
-      <x:c r="B6" s="20"/>
-      <x:c r="C6" s="20"/>
-      <x:c r="D6" s="19" t="str">
+      <x:c r="B6" s="56"/>
+      <x:c r="C6" s="57"/>
+      <x:c r="D6" s="58" t="str">
         <x:f aca="0">IF(OR(B6="",C6=""),"",ROUND(MOD(C6-B6,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E6" s="21"/>
-      <x:c r="F6" s="21"/>
-      <x:c r="G6" s="21"/>
+      <x:c r="E6" s="59"/>
+      <x:c r="F6" s="60"/>
+      <x:c r="G6" s="61"/>
     </x:row>
     <x:row r="7" ht="40" hidden="0" customHeight="1">
-      <x:c r="A7" s="17" t="s">
+      <x:c r="A7" s="62" t="s">
         <x:v>182</x:v>
       </x:c>
-      <x:c r="B7" s="18"/>
-      <x:c r="C7" s="18"/>
-      <x:c r="D7" s="19" t="str">
+      <x:c r="B7" s="63"/>
+      <x:c r="C7" s="64"/>
+      <x:c r="D7" s="65" t="str">
         <x:f aca="0">IF(OR(B7="",C7=""),"",ROUND(MOD(C7-B7,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E7" s="7"/>
-      <x:c r="F7" s="7"/>
-      <x:c r="G7" s="7"/>
+      <x:c r="E7" s="66"/>
+      <x:c r="F7" s="67"/>
+      <x:c r="G7" s="68"/>
     </x:row>
     <x:row r="8" ht="40" hidden="0" customHeight="1">
-      <x:c r="A8" s="17" t="s">
+      <x:c r="A8" s="69" t="s">
         <x:v>182</x:v>
       </x:c>
-      <x:c r="B8" s="20"/>
-      <x:c r="C8" s="20"/>
-      <x:c r="D8" s="19" t="str">
+      <x:c r="B8" s="70"/>
+      <x:c r="C8" s="71"/>
+      <x:c r="D8" s="72" t="str">
         <x:f aca="0">IF(OR(B8="",C8=""),"",ROUND(MOD(C8-B8,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E8" s="21"/>
-      <x:c r="F8" s="21"/>
-      <x:c r="G8" s="21"/>
+      <x:c r="E8" s="73"/>
+      <x:c r="F8" s="74"/>
+      <x:c r="G8" s="75"/>
     </x:row>
     <x:row r="9" ht="40" hidden="0" customHeight="1">
-      <x:c r="A9" s="17" t="s">
+      <x:c r="A9" s="76" t="s">
         <x:v>183</x:v>
       </x:c>
-      <x:c r="B9" s="18"/>
-      <x:c r="C9" s="18"/>
-      <x:c r="D9" s="19" t="str">
+      <x:c r="B9" s="77"/>
+      <x:c r="C9" s="78"/>
+      <x:c r="D9" s="79" t="str">
         <x:f aca="0">IF(OR(B9="",C9=""),"",ROUND(MOD(C9-B9,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E9" s="7"/>
-      <x:c r="F9" s="7"/>
-      <x:c r="G9" s="7"/>
+      <x:c r="E9" s="80"/>
+      <x:c r="F9" s="81"/>
+      <x:c r="G9" s="82"/>
     </x:row>
     <x:row r="10" ht="40" hidden="0" customHeight="1">
-      <x:c r="A10" s="17" t="s">
+      <x:c r="A10" s="83" t="s">
         <x:v>183</x:v>
       </x:c>
-      <x:c r="B10" s="20"/>
-      <x:c r="C10" s="20"/>
-      <x:c r="D10" s="19" t="str">
+      <x:c r="B10" s="84"/>
+      <x:c r="C10" s="85"/>
+      <x:c r="D10" s="86" t="str">
         <x:f aca="0">IF(OR(B10="",C10=""),"",ROUND(MOD(C10-B10,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E10" s="21"/>
-      <x:c r="F10" s="21"/>
-      <x:c r="G10" s="21"/>
+      <x:c r="E10" s="87"/>
+      <x:c r="F10" s="88"/>
+      <x:c r="G10" s="89"/>
     </x:row>
     <x:row r="11" ht="40" hidden="0" customHeight="1">
-      <x:c r="A11" s="17" t="s">
+      <x:c r="A11" s="90" t="s">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="B11" s="18"/>
-      <x:c r="C11" s="18"/>
-      <x:c r="D11" s="19" t="str">
+      <x:c r="B11" s="91"/>
+      <x:c r="C11" s="92"/>
+      <x:c r="D11" s="93" t="str">
         <x:f aca="0">IF(OR(B11="",C11=""),"",ROUND(MOD(C11-B11,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E11" s="7"/>
-      <x:c r="F11" s="7"/>
-      <x:c r="G11" s="7"/>
+      <x:c r="E11" s="94"/>
+      <x:c r="F11" s="95"/>
+      <x:c r="G11" s="96"/>
     </x:row>
     <x:row r="12" ht="40" hidden="0" customHeight="1">
-      <x:c r="A12" s="17" t="s">
+      <x:c r="A12" s="97" t="s">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="B12" s="20"/>
-      <x:c r="C12" s="20"/>
-      <x:c r="D12" s="19" t="str">
+      <x:c r="B12" s="98"/>
+      <x:c r="C12" s="99"/>
+      <x:c r="D12" s="100" t="str">
         <x:f aca="0">IF(OR(B12="",C12=""),"",ROUND(MOD(C12-B12,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E12" s="21"/>
-      <x:c r="F12" s="21"/>
-      <x:c r="G12" s="21"/>
+      <x:c r="E12" s="101"/>
+      <x:c r="F12" s="102"/>
+      <x:c r="G12" s="103"/>
     </x:row>
     <x:row r="13" ht="40" hidden="0" customHeight="1">
-      <x:c r="A13" s="17" t="s">
+      <x:c r="A13" s="104" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="B13" s="18"/>
-      <x:c r="C13" s="18"/>
-      <x:c r="D13" s="19" t="str">
+      <x:c r="B13" s="105"/>
+      <x:c r="C13" s="106"/>
+      <x:c r="D13" s="107" t="str">
         <x:f aca="0">IF(OR(B13="",C13=""),"",ROUND(MOD(C13-B13,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E13" s="7"/>
-      <x:c r="F13" s="7"/>
-      <x:c r="G13" s="7"/>
+      <x:c r="E13" s="108"/>
+      <x:c r="F13" s="109"/>
+      <x:c r="G13" s="110"/>
     </x:row>
     <x:row r="14" ht="40" hidden="0" customHeight="1">
-      <x:c r="A14" s="17" t="s">
+      <x:c r="A14" s="111" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="B14" s="20"/>
-      <x:c r="C14" s="20"/>
-      <x:c r="D14" s="19" t="str">
+      <x:c r="B14" s="112"/>
+      <x:c r="C14" s="113"/>
+      <x:c r="D14" s="114" t="str">
         <x:f aca="0">IF(OR(B14="",C14=""),"",ROUND(MOD(C14-B14,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E14" s="21"/>
-      <x:c r="F14" s="21"/>
-      <x:c r="G14" s="21"/>
+      <x:c r="E14" s="115"/>
+      <x:c r="F14" s="116"/>
+      <x:c r="G14" s="117"/>
     </x:row>
     <x:row r="15" ht="40" hidden="0" customHeight="1">
-      <x:c r="A15" s="17" t="s">
+      <x:c r="A15" s="118" t="s">
         <x:v>186</x:v>
       </x:c>
-      <x:c r="B15" s="18" t="n">
+      <x:c r="B15" s="119" t="n">
         <x:v>0.4375</x:v>
       </x:c>
-      <x:c r="C15" s="18" t="n">
+      <x:c r="C15" s="120" t="n">
         <x:v>0.479166666666667</x:v>
       </x:c>
-      <x:c r="D15" s="19" t="n">
+      <x:c r="D15" s="121" t="n">
         <x:f aca="0">IF(OR(B15="",C15=""),"",ROUND(MOD(C15-B15,1)*1440,6))</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="E15" s="7" t="s">
+      <x:c r="E15" s="122" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="F15" s="7" t="s">
+      <x:c r="F15" s="123" t="s">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="G15" s="7" t="s">
+      <x:c r="G15" s="124" t="s">
         <x:v>187</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="40" hidden="0" customHeight="1">
-      <x:c r="A16" s="17" t="s">
+      <x:c r="A16" s="125" t="s">
         <x:v>186</x:v>
       </x:c>
-      <x:c r="B16" s="20"/>
-      <x:c r="C16" s="20"/>
-      <x:c r="D16" s="19" t="str">
+      <x:c r="B16" s="126"/>
+      <x:c r="C16" s="127"/>
+      <x:c r="D16" s="128" t="str">
         <x:f aca="0">IF(OR(B16="",C16=""),"",ROUND(MOD(C16-B16,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E16" s="21"/>
-      <x:c r="F16" s="21"/>
-      <x:c r="G16" s="21"/>
+      <x:c r="E16" s="129"/>
+      <x:c r="F16" s="130"/>
+      <x:c r="G16" s="131"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Document grouped Daily workbook layout and entry rules
</commit_message>
<xml_diff>
--- a/templates/Training-example.xlsx
+++ b/templates/Training-example.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy" sheetId="1" r:id="Rb82739df4cbe48cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring" sheetId="2" r:id="Rb34766ff17714892"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="3" r:id="R9fb4e1e72596461f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy" sheetId="1" r:id="R9db7c851b401418d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring" sheetId="2" r:id="R116deb64cfce4c61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="3" r:id="Rd22d16428c0e4c68"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -849,7 +849,7 @@
       <x:family val="2"/>
     </x:font>
   </x:fonts>
-  <x:fills count="33">
+  <x:fills count="38">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1011,6 +1011,31 @@
         <x:fgColor rgb="FFF7F9FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F9F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7F9FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4EAF0"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="11">
     <x:border diagonalUp="0" diagonalDown="0">
@@ -1164,7 +1189,7 @@
     <x:xf numFmtId="173" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="174" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="296">
+  <x:cellXfs count="308">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -2207,6 +2232,42 @@
       <x:alignment horizontal="general" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="177" fontId="14" fillId="32" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="176" fontId="15" fillId="33" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="177" fontId="15" fillId="33" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="15" fillId="33" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="176" fontId="15" fillId="34" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="177" fontId="15" fillId="34" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="15" fillId="34" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="177" fontId="15" fillId="35" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="177" fontId="15" fillId="36" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="37" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="26" fillId="37" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="14" fillId="37" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="17" fillId="37" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -4247,7 +4308,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c07be19a62c493a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01a7be38d8d34f14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4266,15 +4327,15 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" hidden="0" customHeight="1">
-      <x:c r="A1" s="181" t="s">
+      <x:c r="A1" s="306" t="s">
         <x:v>181</x:v>
       </x:c>
-      <x:c r="B1" s="181"/>
-      <x:c r="C1" s="181"/>
-      <x:c r="D1" s="181"/>
-      <x:c r="E1" s="181"/>
-      <x:c r="F1" s="181"/>
-      <x:c r="G1" s="185"/>
+      <x:c r="B1" s="306"/>
+      <x:c r="C1" s="306"/>
+      <x:c r="D1" s="306"/>
+      <x:c r="E1" s="306"/>
+      <x:c r="F1" s="306"/>
+      <x:c r="G1" s="307"/>
     </x:row>
     <x:row r="2" ht="28" hidden="0" customHeight="1">
       <x:c r="A2" s="183" t="s">
@@ -4303,49 +4364,49 @@
       <x:c r="A3" s="177" t="s">
         <x:v>188</x:v>
       </x:c>
-      <x:c r="B3" s="285"/>
-      <x:c r="C3" s="285"/>
-      <x:c r="D3" s="197" t="str">
+      <x:c r="B3" s="296"/>
+      <x:c r="C3" s="296"/>
+      <x:c r="D3" s="302" t="str">
         <x:f aca="0">IF(OR(B3="",C3=""),"",ROUND(MOD(C3-B3,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E3" s="278"/>
-      <x:c r="F3" s="278"/>
-      <x:c r="G3" s="278"/>
+      <x:c r="E3" s="298"/>
+      <x:c r="F3" s="298"/>
+      <x:c r="G3" s="298"/>
     </x:row>
     <x:row r="4" ht="26" hidden="0" customHeight="1">
       <x:c r="A4" s="174" t="s">
         <x:v>188</x:v>
       </x:c>
-      <x:c r="B4" s="286"/>
-      <x:c r="C4" s="286"/>
-      <x:c r="D4" s="195" t="str">
+      <x:c r="B4" s="299"/>
+      <x:c r="C4" s="299"/>
+      <x:c r="D4" s="303" t="str">
         <x:f aca="0">IF(OR(B4="",C4=""),"",ROUND(MOD(C4-B4,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E4" s="283"/>
-      <x:c r="F4" s="283"/>
-      <x:c r="G4" s="283"/>
+      <x:c r="E4" s="301"/>
+      <x:c r="F4" s="301"/>
+      <x:c r="G4" s="301"/>
     </x:row>
     <x:row r="5" ht="28" hidden="0" customHeight="1">
       <x:c r="A5" s="177" t="s">
         <x:v>189</x:v>
       </x:c>
-      <x:c r="B5" s="285" t="n">
+      <x:c r="B5" s="296" t="n">
         <x:v>0.833333333333333</x:v>
       </x:c>
-      <x:c r="C5" s="285" t="n">
+      <x:c r="C5" s="296" t="n">
         <x:v>0.875</x:v>
       </x:c>
-      <x:c r="D5" s="197" t="n">
+      <x:c r="D5" s="302" t="n">
         <x:f aca="0">IF(OR(B5="",C5=""),"",ROUND(MOD(C5-B5,1)*1440,6))</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="E5" s="278" t="s">
+      <x:c r="E5" s="298" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="F5" s="278" t="s">
+      <x:c r="F5" s="298" t="s">
         <x:v>190</x:v>
       </x:c>
-      <x:c r="G5" s="278" t="s">
+      <x:c r="G5" s="298" t="s">
         <x:v>191</x:v>
       </x:c>
     </x:row>
@@ -4353,140 +4414,140 @@
       <x:c r="A6" s="174" t="s">
         <x:v>189</x:v>
       </x:c>
-      <x:c r="B6" s="286"/>
-      <x:c r="C6" s="286"/>
-      <x:c r="D6" s="195" t="str">
+      <x:c r="B6" s="299"/>
+      <x:c r="C6" s="299"/>
+      <x:c r="D6" s="303" t="str">
         <x:f aca="0">IF(OR(B6="",C6=""),"",ROUND(MOD(C6-B6,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E6" s="283"/>
-      <x:c r="F6" s="283"/>
-      <x:c r="G6" s="283"/>
+      <x:c r="E6" s="301"/>
+      <x:c r="F6" s="301"/>
+      <x:c r="G6" s="301"/>
     </x:row>
     <x:row r="7" ht="26" hidden="0" customHeight="1">
       <x:c r="A7" s="177" t="s">
         <x:v>192</x:v>
       </x:c>
-      <x:c r="B7" s="285"/>
-      <x:c r="C7" s="285"/>
-      <x:c r="D7" s="197" t="str">
+      <x:c r="B7" s="296"/>
+      <x:c r="C7" s="296"/>
+      <x:c r="D7" s="302" t="str">
         <x:f aca="0">IF(OR(B7="",C7=""),"",ROUND(MOD(C7-B7,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E7" s="278"/>
-      <x:c r="F7" s="278"/>
-      <x:c r="G7" s="278"/>
+      <x:c r="E7" s="298"/>
+      <x:c r="F7" s="298"/>
+      <x:c r="G7" s="298"/>
     </x:row>
     <x:row r="8" ht="26" hidden="0" customHeight="1">
       <x:c r="A8" s="174" t="s">
         <x:v>192</x:v>
       </x:c>
-      <x:c r="B8" s="286"/>
-      <x:c r="C8" s="286"/>
-      <x:c r="D8" s="195" t="str">
+      <x:c r="B8" s="299"/>
+      <x:c r="C8" s="299"/>
+      <x:c r="D8" s="303" t="str">
         <x:f aca="0">IF(OR(B8="",C8=""),"",ROUND(MOD(C8-B8,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E8" s="283"/>
-      <x:c r="F8" s="283"/>
-      <x:c r="G8" s="283"/>
+      <x:c r="E8" s="301"/>
+      <x:c r="F8" s="301"/>
+      <x:c r="G8" s="301"/>
     </x:row>
     <x:row r="9" ht="26" hidden="0" customHeight="1">
       <x:c r="A9" s="177" t="s">
         <x:v>193</x:v>
       </x:c>
-      <x:c r="B9" s="285"/>
-      <x:c r="C9" s="285"/>
-      <x:c r="D9" s="197" t="str">
+      <x:c r="B9" s="296"/>
+      <x:c r="C9" s="296"/>
+      <x:c r="D9" s="302" t="str">
         <x:f aca="0">IF(OR(B9="",C9=""),"",ROUND(MOD(C9-B9,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E9" s="278"/>
-      <x:c r="F9" s="278"/>
-      <x:c r="G9" s="278"/>
+      <x:c r="E9" s="298"/>
+      <x:c r="F9" s="298"/>
+      <x:c r="G9" s="298"/>
     </x:row>
     <x:row r="10" ht="26" hidden="0" customHeight="1">
       <x:c r="A10" s="174" t="s">
         <x:v>193</x:v>
       </x:c>
-      <x:c r="B10" s="286"/>
-      <x:c r="C10" s="286"/>
-      <x:c r="D10" s="195" t="str">
+      <x:c r="B10" s="299"/>
+      <x:c r="C10" s="299"/>
+      <x:c r="D10" s="303" t="str">
         <x:f aca="0">IF(OR(B10="",C10=""),"",ROUND(MOD(C10-B10,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E10" s="283"/>
-      <x:c r="F10" s="283"/>
-      <x:c r="G10" s="283"/>
+      <x:c r="E10" s="301"/>
+      <x:c r="F10" s="301"/>
+      <x:c r="G10" s="301"/>
     </x:row>
     <x:row r="11" ht="26" hidden="0" customHeight="1">
       <x:c r="A11" s="177" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="B11" s="285"/>
-      <x:c r="C11" s="285"/>
-      <x:c r="D11" s="197" t="str">
+      <x:c r="B11" s="296"/>
+      <x:c r="C11" s="296"/>
+      <x:c r="D11" s="302" t="str">
         <x:f aca="0">IF(OR(B11="",C11=""),"",ROUND(MOD(C11-B11,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E11" s="278"/>
-      <x:c r="F11" s="278"/>
-      <x:c r="G11" s="278"/>
+      <x:c r="E11" s="298"/>
+      <x:c r="F11" s="298"/>
+      <x:c r="G11" s="298"/>
     </x:row>
     <x:row r="12" ht="26" hidden="0" customHeight="1">
       <x:c r="A12" s="174" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="B12" s="286"/>
-      <x:c r="C12" s="286"/>
-      <x:c r="D12" s="195" t="str">
+      <x:c r="B12" s="299"/>
+      <x:c r="C12" s="299"/>
+      <x:c r="D12" s="303" t="str">
         <x:f aca="0">IF(OR(B12="",C12=""),"",ROUND(MOD(C12-B12,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E12" s="283"/>
-      <x:c r="F12" s="283"/>
-      <x:c r="G12" s="283"/>
+      <x:c r="E12" s="301"/>
+      <x:c r="F12" s="301"/>
+      <x:c r="G12" s="301"/>
     </x:row>
     <x:row r="13" ht="26" hidden="0" customHeight="1">
       <x:c r="A13" s="177" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="B13" s="285"/>
-      <x:c r="C13" s="285"/>
-      <x:c r="D13" s="197" t="str">
+      <x:c r="B13" s="296"/>
+      <x:c r="C13" s="296"/>
+      <x:c r="D13" s="302" t="str">
         <x:f aca="0">IF(OR(B13="",C13=""),"",ROUND(MOD(C13-B13,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E13" s="278"/>
-      <x:c r="F13" s="278"/>
-      <x:c r="G13" s="278"/>
+      <x:c r="E13" s="298"/>
+      <x:c r="F13" s="298"/>
+      <x:c r="G13" s="298"/>
     </x:row>
     <x:row r="14" ht="26" hidden="0" customHeight="1">
       <x:c r="A14" s="174" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="B14" s="286"/>
-      <x:c r="C14" s="286"/>
-      <x:c r="D14" s="195" t="str">
+      <x:c r="B14" s="299"/>
+      <x:c r="C14" s="299"/>
+      <x:c r="D14" s="303" t="str">
         <x:f aca="0">IF(OR(B14="",C14=""),"",ROUND(MOD(C14-B14,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E14" s="283"/>
-      <x:c r="F14" s="283"/>
-      <x:c r="G14" s="283"/>
+      <x:c r="E14" s="301"/>
+      <x:c r="F14" s="301"/>
+      <x:c r="G14" s="301"/>
     </x:row>
     <x:row r="15" ht="28" hidden="0" customHeight="1">
       <x:c r="A15" s="177" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="B15" s="285" t="n">
+      <x:c r="B15" s="296" t="n">
         <x:v>0.4375</x:v>
       </x:c>
-      <x:c r="C15" s="285" t="n">
+      <x:c r="C15" s="296" t="n">
         <x:v>0.479166666666667</x:v>
       </x:c>
-      <x:c r="D15" s="197" t="n">
+      <x:c r="D15" s="302" t="n">
         <x:f aca="0">IF(OR(B15="",C15=""),"",ROUND(MOD(C15-B15,1)*1440,6))</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="E15" s="278" t="s">
+      <x:c r="E15" s="298" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="F15" s="278" t="s">
+      <x:c r="F15" s="298" t="s">
         <x:v>190</x:v>
       </x:c>
-      <x:c r="G15" s="278" t="s">
+      <x:c r="G15" s="298" t="s">
         <x:v>197</x:v>
       </x:c>
     </x:row>
@@ -4494,14 +4555,14 @@
       <x:c r="A16" s="174" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="B16" s="286"/>
-      <x:c r="C16" s="286"/>
-      <x:c r="D16" s="195" t="str">
+      <x:c r="B16" s="299"/>
+      <x:c r="C16" s="299"/>
+      <x:c r="D16" s="303" t="str">
         <x:f aca="0">IF(OR(B16="",C16=""),"",ROUND(MOD(C16-B16,1)*1440,6))</x:f>
       </x:c>
-      <x:c r="E16" s="283"/>
-      <x:c r="F16" s="283"/>
-      <x:c r="G16" s="283"/>
+      <x:c r="E16" s="301"/>
+      <x:c r="F16" s="301"/>
+      <x:c r="G16" s="301"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>